<commit_message>
Fix generate excel column and update report_summary
</commit_message>
<xml_diff>
--- a/CoursePatterns/Output/course_frequency.xlsx
+++ b/CoursePatterns/Output/course_frequency.xlsx
@@ -549,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -571,37 +571,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>COSE214</t>
+          <t>COSE213</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>COSE341</t>
+          <t>COSE214</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>COSE222</t>
+          <t>COSE341</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>COSE211</t>
+          <t>COSE222</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -611,37 +611,37 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>COSE342</t>
+          <t>COSE211</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>COSE221</t>
+          <t>COSE342</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>COSE371</t>
+          <t>COSE221</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>COSE215</t>
+          <t>COSE371</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -651,77 +651,77 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>COSE361</t>
+          <t>COSE215</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>COSE281</t>
+          <t>COSE361</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>COSE474</t>
+          <t>COSE281</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>COSE212</t>
+          <t>COSE474</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>COSE471</t>
+          <t>COSE212</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>COSE382</t>
+          <t>COSE471</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>COSE352</t>
+          <t>COSE382</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>COSE312</t>
+          <t>COSE352</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -731,17 +731,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>COSE362</t>
+          <t>COSE312</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>COSE242</t>
+          <t>COSE362</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -751,7 +751,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>COSE461</t>
+          <t>COSE242</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -761,17 +761,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>COSE389</t>
+          <t>COSE461</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>COSE385</t>
+          <t>COSE389</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -781,7 +781,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>COSE284</t>
+          <t>COSE385</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -791,17 +791,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>COSE331</t>
+          <t>COSE284</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>COSE283</t>
+          <t>COSE331</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -811,7 +811,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>COSE322</t>
+          <t>COSE283</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -821,7 +821,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>COSE354</t>
+          <t>COSE322</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -831,7 +831,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>COSE490</t>
+          <t>COSE354</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -841,7 +841,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>COSE441</t>
+          <t>COSE490</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -851,17 +851,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>COSE455</t>
+          <t>COSE441</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>COSE421</t>
+          <t>COSE455</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -871,17 +871,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>COSE372</t>
+          <t>COSE421</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>COSE321</t>
+          <t>COSE372</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -891,7 +891,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>COSE405</t>
+          <t>COSE321</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -901,7 +901,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>COSE423</t>
+          <t>COSE405</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -911,7 +911,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>COSE483</t>
+          <t>COSE423</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -921,17 +921,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>COSE485</t>
+          <t>COSE483</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>COSE415</t>
+          <t>COSE485</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -941,7 +941,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>COSE432</t>
+          <t>COSE415</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -951,7 +951,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>COSE363</t>
+          <t>COSE432</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -961,17 +961,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>COSE451</t>
+          <t>COSE363</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>DATA303</t>
+          <t>COSE451</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -981,7 +981,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>COSE484</t>
+          <t>DATA303</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -991,7 +991,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>DATA403</t>
+          <t>COSE484</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1001,7 +1001,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>COSE380</t>
+          <t>DATA403</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1011,7 +1011,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>COSE444</t>
+          <t>COSE380</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1021,7 +1021,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>COSE436</t>
+          <t>COSE444</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1031,17 +1031,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>COSE407</t>
+          <t>COSE436</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>COSE394</t>
+          <t>COSE407</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1051,10 +1051,20 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>COSE394</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>COSE457</t>
         </is>
       </c>
-      <c r="B50" t="n">
+      <c r="B51" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>